<commit_message>
feat: Rebuild 5 BRD Excel - pure business language, no technical DD content
</commit_message>
<xml_diff>
--- a/2. Tài liệu phân tích và thiết kế/02. BRD & Template/BRD_Excel/1_BRD_Doanh_Thu_Cong_Ty.xlsx
+++ b/2. Tài liệu phân tích và thiết kế/02. BRD & Template/BRD_Excel/1_BRD_Doanh_Thu_Cong_Ty.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +27,42 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -42,8 +71,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-        <bgColor rgb="00D9D9D9"/>
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,20 +109,46 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -436,258 +515,817 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TÀI LIỆU YÊU CẦU NGHIỆP VỤ (BRD) - BÁO CÁO DOANH THU CỦA CÔNG TY</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+          <t>BRD 1 - BÁO CÁO DOANH THU CÔNG TY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="6" customHeight="1"/>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Ghi chú: Xây dựng báo cáo trên hệ thống báo cáo tập trung Power BI.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>1. Mục đích báo cáo</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>- Xây dựng: BÁO CÁO DOANH THU CỦA CÔNG TY</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Báo cáo doanh thu tổng quan của toàn công ty Sovigaz</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2. Nội dung báo cáo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>2.1. Nguồn dữ liệu</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Nguồn dữ liệu</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Mô tả luồng xử lý</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Thời gian Data sẵn sàng</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Thời điểm lấy dữ liệu</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Phần mềm kế toán MISA</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Đồng bộ dữ liệu từ MISA -&gt; Database -&gt; DWH.Staging -&gt; DWH.DWH -&gt; DWH.DM -&gt; Báo cáo</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Dữ liệu doanh thu theo sản phẩm, xí nghiệp</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>9h30 AM</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Từ năm 2018 đến hiện tại</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Thông tin đối chiếu</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Đối chiếu từ MISA</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Danh mục khách hàng MISA</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Thông tin phân loại nhóm khách hàng</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>9h30 AM</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Từ năm 2018 đến hiện tại</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Danh mục kho/chi nhánh MISA</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Tên xí nghiệp, chi nhánh</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>9h30 AM</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Từ năm 2018 đến hiện tại</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>2.2. Điều kiện ràng buộc xuyên suốt báo cáo</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Điều kiện</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="E13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="4" t="inlineStr"/>
-      <c r="E14" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Phân biệt doanh thu bán ngoài và nội bộ</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Doanh thu bán ngoài là doanh thu từ khách hàng bên ngoài công ty. Doanh thu LCNB là doanh thu luân chuyển nội bộ giữa các xí nghiệp</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Đơn vị tiền tệ</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Tất cả các giá trị tiền tệ hiển thị bằng VNĐ</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>2.3. Filter báo cáo</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Bộ lọc</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Mô tả</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Giá trị mẫu/Định dạng</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Đặc tính</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="4" t="inlineStr"/>
-      <c r="E18" s="4" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Khoảng thời gian (Từ ngày - Đến ngày)</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Lọc dữ liệu theo khoảng thời gian phát sinh doanh thu</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Ngày/Tháng/Năm</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Tên khách hàng</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Tìm kiếm/lọc theo tên khách hàng cụ thể</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Dropdown / Search</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Tên nhóm khách hàng</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Lọc theo nhóm phân loại khách hàng (Bệnh viện, Đại lý, Công nghiệp...)</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Dropdown</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Tên xí nghiệp</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Lọc theo xí nghiệp/chi nhánh trực thuộc Sovigaz</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Dropdown</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Tên sản phẩm</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Tìm kiếm doanh thu theo tên sản phẩm/mặt hàng</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Search (gõ để tìm)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>2.4. Chi tiết các trường dữ liệu (Metrics/Dimensions)</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Chỉ tiêu</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Mô tả/Cách tính</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Mô tả / Nghiệp vụ tính toán</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Loại dữ liệu</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Đơn vị</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Biểu đồ</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr"/>
-      <c r="B22" s="4" t="inlineStr"/>
-      <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="4" t="inlineStr"/>
-      <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>CARD</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Doanh thu bán ngoài</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Tổng doanh thu từ tất cả khách hàng bên ngoài công ty trong kỳ được chọn</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>VNĐ</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Doanh thu LCNB</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Tổng doanh thu luân chuyển nội bộ giữa các xí nghiệp trực thuộc Sovigaz</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>VNĐ</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr"/>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Tổng số đơn hàng</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Tổng số đơn hàng/hóa đơn phát sinh trong kỳ</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Số nguyên</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>Đơn</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Giá trị trung bình của đơn hàng</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Doanh thu bán ngoài chia cho tổng số đơn hàng</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>VNĐ</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>CHART</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="10" t="n"/>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="10" t="n"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Doanh thu và số đơn hàng theo tháng</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Biểu đồ kết hợp cột và đường thể hiện doanh thu (cột) và số đơn hàng (đường) theo từng tháng trong năm</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Số tiền / Số nguyên</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>VNĐ / Đơn</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Line and Stacked Column Chart</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Doanh thu theo nhóm vật tư, hàng hóa</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Biểu đồ cột chồng thể hiện doanh thu phân theo nhóm sản phẩm (khí công nghiệp, que hàn, hóa chất...)</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>VNĐ</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Stacked Column Chart</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr"/>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Doanh thu theo tháng của nhóm khách hàng</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Biểu đồ cột nhóm thể hiện doanh thu theo tháng, phân tách theo nhóm khách hàng</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>VNĐ</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Clustered Column Chart</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Tỷ lệ đóng góp doanh thu theo nhóm khách hàng</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Biểu đồ tròn thể hiện % đóng góp doanh thu của từng nhóm khách hàng</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Tỷ lệ</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Pie Chart</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Doanh thu theo tháng của xí nghiệp</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Biểu đồ cột chồng thể hiện doanh thu theo tháng, phân tách theo từng xí nghiệp</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Số tiền</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>VNĐ</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Stacked Column Chart</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Tỷ lệ đóng góp doanh thu theo xí nghiệp</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Biểu đồ tròn thể hiện % đóng góp doanh thu của từng xí nghiệp trên tổng doanh thu</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Tỷ lệ</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Pie Chart</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A6:H6"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>